<commit_message>
Fix RTL number display in summary tables
</commit_message>
<xml_diff>
--- a/analysis_outputs/tables/event_study_panel_summary_baseline_minus1.xlsx
+++ b/analysis_outputs/tables/event_study_panel_summary_baseline_minus1.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event Study" sheetId="1" r:id="R1abe62dce28440d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event Study" sheetId="1" r:id="R21f0ca2534644e77"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -301,35 +301,35 @@
         <x:v>המשתנה התלוי: log(הוצאה שבועית)</x:v>
       </x:c>
       <x:c r="B1" s="8" t="str">
-        <x:v>(1) כל המפרסמים</x:v>
+        <x:v>‎(1) כל המפרסמים</x:v>
       </x:c>
       <x:c r="C1" s="8" t="str">
-        <x:v>(2) מפלגות</x:v>
+        <x:v>‎(2) מפלגות</x:v>
       </x:c>
       <x:c r="D1" s="8" t="str">
-        <x:v>(3) גופים פרטיים</x:v>
+        <x:v>‎(3) גופים פרטיים</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="12" t="str">
         <x:v>פאנל א': כל האירועים</x:v>
       </x:c>
-      <x:c r="B2" s="12" t="str"/>
-      <x:c r="C2" s="12" t="str"/>
-      <x:c r="D2" s="12" t="str"/>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="15" t="str">
         <x:v>מקדם שבוע +1 (β)</x:v>
       </x:c>
       <x:c r="B3" s="5" t="str">
-        <x:v>-0.081***</x:v>
+        <x:v>‎-0.081***</x:v>
       </x:c>
       <x:c r="C3" s="5" t="str">
-        <x:v>-0.091</x:v>
+        <x:v>‎-0.091</x:v>
       </x:c>
       <x:c r="D3" s="5" t="str">
-        <x:v>-0.057**</x:v>
+        <x:v>‎-0.057**</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -337,35 +337,35 @@
         <x:v>(טעות תקן)</x:v>
       </x:c>
       <x:c r="B4" s="13" t="str">
-        <x:v>(0.027)</x:v>
+        <x:v>‎(0.027)</x:v>
       </x:c>
       <x:c r="C4" s="13" t="str">
-        <x:v>(0.101)</x:v>
+        <x:v>‎(0.101)</x:v>
       </x:c>
       <x:c r="D4" s="13" t="str">
-        <x:v>(0.027)</x:v>
+        <x:v>‎(0.027)</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
         <x:v>פאנל ב': אירועים פוליטיים</x:v>
       </x:c>
-      <x:c r="B5" s="12" t="str"/>
-      <x:c r="C5" s="12" t="str"/>
-      <x:c r="D5" s="12" t="str"/>
+      <x:c r="B5" s="11"/>
+      <x:c r="C5" s="11"/>
+      <x:c r="D5" s="11"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="15" t="str">
         <x:v>מקדם שבוע +1 (β)</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>-0.215***</x:v>
+        <x:v>‎-0.215***</x:v>
       </x:c>
       <x:c r="C6" s="5" t="str">
-        <x:v>-0.359</x:v>
+        <x:v>‎-0.359</x:v>
       </x:c>
       <x:c r="D6" s="5" t="str">
-        <x:v>-0.164***</x:v>
+        <x:v>‎-0.164***</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -373,35 +373,35 @@
         <x:v>(טעות תקן)</x:v>
       </x:c>
       <x:c r="B7" s="13" t="str">
-        <x:v>(0.047)</x:v>
+        <x:v>‎(0.047)</x:v>
       </x:c>
       <x:c r="C7" s="13" t="str">
-        <x:v>(0.228)</x:v>
+        <x:v>‎(0.228)</x:v>
       </x:c>
       <x:c r="D7" s="13" t="str">
-        <x:v>(0.044)</x:v>
+        <x:v>‎(0.044)</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
         <x:v>פאנל ג': אירועי טרור</x:v>
       </x:c>
-      <x:c r="B8" s="12" t="str"/>
-      <x:c r="C8" s="12" t="str"/>
-      <x:c r="D8" s="12" t="str"/>
+      <x:c r="B8" s="11"/>
+      <x:c r="C8" s="11"/>
+      <x:c r="D8" s="11"/>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="15" t="str">
         <x:v>מקדם שבוע +1 (β)</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>0.075*</x:v>
+        <x:v>‎0.075*</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
-        <x:v>0.174*</x:v>
+        <x:v>‎0.174*</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
-        <x:v>0.069*</x:v>
+        <x:v>‎0.069*</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -409,35 +409,35 @@
         <x:v>(טעות תקן)</x:v>
       </x:c>
       <x:c r="B10" s="13" t="str">
-        <x:v>(0.038)</x:v>
+        <x:v>‎(0.038)</x:v>
       </x:c>
       <x:c r="C10" s="13" t="str">
-        <x:v>(0.085)</x:v>
+        <x:v>‎(0.085)</x:v>
       </x:c>
       <x:c r="D10" s="13" t="str">
-        <x:v>(0.039)</x:v>
+        <x:v>‎(0.039)</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
         <x:v>בקרות ונתוני מודל</x:v>
       </x:c>
-      <x:c r="B11" s="12" t="str"/>
-      <x:c r="C11" s="12" t="str"/>
-      <x:c r="D11" s="12" t="str"/>
+      <x:c r="B11" s="11"/>
+      <x:c r="C11" s="11"/>
+      <x:c r="D11" s="11"/>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="15" t="str">
         <x:v>R2 - כל האירועים</x:v>
       </x:c>
       <x:c r="B12" s="5" t="str">
-        <x:v>0.347</x:v>
+        <x:v>‎0.347</x:v>
       </x:c>
       <x:c r="C12" s="5" t="str">
-        <x:v>0.436</x:v>
+        <x:v>‎0.436</x:v>
       </x:c>
       <x:c r="D12" s="5" t="str">
-        <x:v>0.362</x:v>
+        <x:v>‎0.362</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -445,13 +445,13 @@
         <x:v>R2 - אירועים פוליטיים</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
-        <x:v>0.329</x:v>
+        <x:v>‎0.329</x:v>
       </x:c>
       <x:c r="C13" s="5" t="str">
-        <x:v>0.454</x:v>
+        <x:v>‎0.454</x:v>
       </x:c>
       <x:c r="D13" s="5" t="str">
-        <x:v>0.342</x:v>
+        <x:v>‎0.342</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -459,13 +459,13 @@
         <x:v>R2 - אירועי טרור</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>0.407</x:v>
+        <x:v>‎0.407</x:v>
       </x:c>
       <x:c r="C14" s="5" t="str">
-        <x:v>0.483</x:v>
+        <x:v>‎0.483</x:v>
       </x:c>
       <x:c r="D14" s="5" t="str">
-        <x:v>0.415</x:v>
+        <x:v>‎0.415</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -487,13 +487,13 @@
         <x:v>N - כל האירועים</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>10038</x:v>
+        <x:v>‎10038</x:v>
       </x:c>
       <x:c r="C16" s="5" t="str">
-        <x:v>1411</x:v>
+        <x:v>‎1411</x:v>
       </x:c>
       <x:c r="D16" s="5" t="str">
-        <x:v>8627</x:v>
+        <x:v>‎8627</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -501,13 +501,13 @@
         <x:v>N - אירועים פוליטיים</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
-        <x:v>5323</x:v>
+        <x:v>‎5323</x:v>
       </x:c>
       <x:c r="C17" s="5" t="str">
-        <x:v>755</x:v>
+        <x:v>‎755</x:v>
       </x:c>
       <x:c r="D17" s="5" t="str">
-        <x:v>4568</x:v>
+        <x:v>‎4568</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -515,13 +515,13 @@
         <x:v>N - אירועי טרור</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>4714</x:v>
+        <x:v>‎4714</x:v>
       </x:c>
       <x:c r="C18" s="5" t="str">
-        <x:v>656</x:v>
+        <x:v>‎656</x:v>
       </x:c>
       <x:c r="D18" s="5" t="str">
-        <x:v>4058</x:v>
+        <x:v>‎4058</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>